<commit_message>
Adjust changes in postprocessing
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_cost_factors/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_cost_factors/cb_config_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_uganda_data/ssp_modeling/cost-benefits/cb_cost_factors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_uganda_data/ssp_modeling/cost-benefits/cb_cost_factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45F9F33-4552-1144-8775-D6585E62E627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D86C61C-F8CB-E04E-A4D4-C192C37F0926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30780" yWindow="-7160" windowWidth="30780" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30780" yWindow="-9740" windowWidth="30780" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
     <sheet name="attribute_transformation_code" sheetId="17" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">cost_factors!$A$1:$L$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">cost_factors!$A$1:$L$162</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4783" uniqueCount="2057">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4835" uniqueCount="2067">
   <si>
     <t>output_variable_name</t>
   </si>
@@ -6250,6 +6250,36 @@
   </si>
   <si>
     <t>cb:entc:technical_savings:electricity:opex</t>
+  </si>
+  <si>
+    <t>cb:lndu:technical_cost:grasslands:X</t>
+  </si>
+  <si>
+    <t>cb:lndu:ecosystem_services_grasslands:grasslands:X</t>
+  </si>
+  <si>
+    <t>cb:lndu:ecosystem_services_wetlands:wetlands:X</t>
+  </si>
+  <si>
+    <t>cb:lndu:technical_cost:wetlands:X</t>
+  </si>
+  <si>
+    <t>area_lndu_wetlands</t>
+  </si>
+  <si>
+    <t>area_lndu_grasslands</t>
+  </si>
+  <si>
+    <t>Benefits wetlands</t>
+  </si>
+  <si>
+    <t>Cost of Maintenance</t>
+  </si>
+  <si>
+    <t>Benefits grasslands</t>
+  </si>
+  <si>
+    <t>Alexa added this</t>
   </si>
 </sst>
 </file>
@@ -6387,7 +6417,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -6690,7 +6720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E217"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="59" bestFit="1" customWidth="1"/>
@@ -10313,6 +10343,62 @@
       </c>
       <c r="E213" s="5" t="s">
         <v>434</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A214" s="3" t="s">
+        <v>2059</v>
+      </c>
+      <c r="B214" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C214" s="5" t="s">
+        <v>2066</v>
+      </c>
+      <c r="E214" s="5" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A215" s="3" t="s">
+        <v>2060</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C215" s="5" t="s">
+        <v>2066</v>
+      </c>
+      <c r="E215" s="5" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A216" s="3" t="s">
+        <v>2058</v>
+      </c>
+      <c r="B216" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C216" s="5" t="s">
+        <v>2066</v>
+      </c>
+      <c r="E216" s="5" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A217" s="3" t="s">
+        <v>2057</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>2066</v>
+      </c>
+      <c r="E217" s="5" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -16846,7 +16932,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L159"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
@@ -20011,205 +20097,205 @@
         <v>693</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>115</v>
-      </c>
-      <c r="B84" t="s">
-        <v>535</v>
-      </c>
-      <c r="C84">
-        <v>323.52941179999999</v>
-      </c>
-      <c r="D84" t="s">
-        <v>591</v>
-      </c>
-      <c r="E84">
-        <v>1</v>
-      </c>
-      <c r="F84" t="s">
-        <v>265</v>
-      </c>
-      <c r="G84" t="b">
-        <v>1</v>
-      </c>
-      <c r="H84" t="s">
-        <v>675</v>
-      </c>
-      <c r="I84" t="s">
+    <row r="84" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>2059</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>2061</v>
+      </c>
+      <c r="C84" s="3">
+        <v>30373</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="E84" s="3">
+        <v>1</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>2063</v>
+      </c>
+      <c r="G84" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="J84" t="s">
-        <v>357</v>
-      </c>
-      <c r="K84" t="s">
+      <c r="I84" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J84" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K84" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L84" t="s">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>37</v>
-      </c>
-      <c r="B85" t="s">
-        <v>476</v>
-      </c>
-      <c r="C85">
-        <v>260</v>
-      </c>
-      <c r="D85" t="s">
-        <v>589</v>
-      </c>
-      <c r="E85">
-        <v>1</v>
-      </c>
-      <c r="F85" t="s">
-        <v>243</v>
-      </c>
-      <c r="G85" t="b">
+      <c r="L84" s="3" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>2060</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>2061</v>
+      </c>
+      <c r="C85" s="3">
+        <v>-135</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="E85" s="3">
+        <v>1</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>2064</v>
+      </c>
+      <c r="G85" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H85" t="s">
-        <v>624</v>
-      </c>
-      <c r="I85" t="s">
-        <v>678</v>
-      </c>
-      <c r="J85" t="s">
-        <v>352</v>
-      </c>
-      <c r="K85" t="s">
+      <c r="H85" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J85" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K85" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L85" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>38</v>
-      </c>
-      <c r="B86" t="s">
-        <v>477</v>
-      </c>
-      <c r="C86">
-        <v>260</v>
-      </c>
-      <c r="D86" t="s">
-        <v>589</v>
-      </c>
-      <c r="E86">
-        <v>1</v>
-      </c>
-      <c r="F86" t="s">
-        <v>244</v>
-      </c>
-      <c r="G86" t="b">
+      <c r="L85" s="3" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>2058</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>2062</v>
+      </c>
+      <c r="C86" s="3">
+        <v>5700</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="E86" s="3">
+        <v>1</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>2065</v>
+      </c>
+      <c r="G86" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H86" t="s">
-        <v>624</v>
-      </c>
-      <c r="I86" t="s">
-        <v>678</v>
-      </c>
-      <c r="J86" t="s">
-        <v>352</v>
-      </c>
-      <c r="K86" t="s">
+      <c r="H86" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J86" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K86" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L86" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>39</v>
-      </c>
-      <c r="B87" t="s">
-        <v>478</v>
-      </c>
-      <c r="C87">
-        <v>260</v>
-      </c>
-      <c r="D87" t="s">
-        <v>589</v>
-      </c>
-      <c r="E87">
-        <v>1</v>
-      </c>
-      <c r="F87" t="s">
-        <v>245</v>
-      </c>
-      <c r="G87" t="b">
+      <c r="L86" s="3" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>2057</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>2062</v>
+      </c>
+      <c r="C87" s="3">
+        <v>-77.69</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="E87" s="3">
+        <v>1</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>2064</v>
+      </c>
+      <c r="G87" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H87" t="s">
-        <v>624</v>
-      </c>
-      <c r="I87" t="s">
-        <v>678</v>
-      </c>
-      <c r="J87" t="s">
-        <v>352</v>
-      </c>
-      <c r="K87" t="s">
+      <c r="H87" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="J87" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K87" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L87" t="s">
-        <v>698</v>
+      <c r="L87" s="3" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>40</v>
+        <v>115</v>
       </c>
       <c r="B88" t="s">
-        <v>479</v>
+        <v>535</v>
       </c>
       <c r="C88">
-        <v>2.6</v>
+        <v>323.52941179999999</v>
       </c>
       <c r="D88" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E88">
         <v>1</v>
       </c>
       <c r="F88" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="G88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H88" t="s">
-        <v>625</v>
+        <v>675</v>
       </c>
       <c r="I88" t="s">
-        <v>678</v>
+        <v>349</v>
       </c>
       <c r="J88" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="K88" t="s">
         <v>687</v>
       </c>
       <c r="L88" t="s">
-        <v>698</v>
+        <v>715</v>
       </c>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B89" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="C89">
-        <v>26</v>
+        <v>260</v>
       </c>
       <c r="D89" t="s">
         <v>589</v>
@@ -20218,13 +20304,13 @@
         <v>1</v>
       </c>
       <c r="F89" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="G89" t="b">
         <v>0</v>
       </c>
       <c r="H89" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="I89" t="s">
         <v>678</v>
@@ -20241,13 +20327,13 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B90" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="C90">
-        <v>200</v>
+        <v>260</v>
       </c>
       <c r="D90" t="s">
         <v>589</v>
@@ -20256,13 +20342,13 @@
         <v>1</v>
       </c>
       <c r="F90" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="G90" t="b">
         <v>0</v>
       </c>
       <c r="H90" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I90" t="s">
         <v>678</v>
@@ -20279,13 +20365,13 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="C91">
-        <v>200</v>
+        <v>260</v>
       </c>
       <c r="D91" t="s">
         <v>589</v>
@@ -20294,13 +20380,13 @@
         <v>1</v>
       </c>
       <c r="F91" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="G91" t="b">
         <v>0</v>
       </c>
       <c r="H91" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I91" t="s">
         <v>678</v>
@@ -20317,13 +20403,13 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B92" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="C92">
-        <v>50</v>
+        <v>2.6</v>
       </c>
       <c r="D92" t="s">
         <v>589</v>
@@ -20332,13 +20418,13 @@
         <v>1</v>
       </c>
       <c r="F92" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G92" t="b">
         <v>0</v>
       </c>
       <c r="H92" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="I92" t="s">
         <v>678</v>
@@ -20355,10 +20441,10 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B93" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="C93">
         <v>26</v>
@@ -20370,7 +20456,7 @@
         <v>1</v>
       </c>
       <c r="F93" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="G93" t="b">
         <v>0</v>
@@ -20393,297 +20479,297 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="B94" t="s">
-        <v>514</v>
+        <v>481</v>
       </c>
       <c r="C94">
-        <v>-1000000</v>
+        <v>200</v>
       </c>
       <c r="D94" t="s">
-        <v>349</v>
+        <v>589</v>
       </c>
       <c r="E94">
         <v>1</v>
       </c>
       <c r="F94" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="G94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H94" t="s">
-        <v>349</v>
+        <v>627</v>
       </c>
       <c r="I94" t="s">
-        <v>393</v>
+        <v>678</v>
       </c>
       <c r="J94" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="K94" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L94" t="s">
-        <v>705</v>
+        <v>698</v>
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A95" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>501</v>
-      </c>
-      <c r="C95" s="3">
-        <v>-500</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="E95" s="3">
-        <v>1</v>
-      </c>
-      <c r="F95" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="G95" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H95" s="3" t="s">
-        <v>641</v>
-      </c>
-      <c r="I95" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="J95" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="K95" s="3" t="s">
+      <c r="A95" t="s">
+        <v>43</v>
+      </c>
+      <c r="B95" t="s">
+        <v>482</v>
+      </c>
+      <c r="C95">
+        <v>200</v>
+      </c>
+      <c r="D95" t="s">
+        <v>589</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95" t="s">
+        <v>249</v>
+      </c>
+      <c r="G95" t="b">
+        <v>0</v>
+      </c>
+      <c r="H95" t="s">
+        <v>627</v>
+      </c>
+      <c r="I95" t="s">
+        <v>678</v>
+      </c>
+      <c r="J95" t="s">
+        <v>352</v>
+      </c>
+      <c r="K95" t="s">
         <v>687</v>
       </c>
-      <c r="L95" s="3" t="s">
-        <v>700</v>
+      <c r="L95" t="s">
+        <v>698</v>
       </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>99</v>
+        <v>44</v>
       </c>
       <c r="B96" t="s">
-        <v>523</v>
+        <v>483</v>
       </c>
       <c r="C96">
-        <v>-60000</v>
+        <v>50</v>
       </c>
       <c r="D96" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
       <c r="E96">
         <v>1</v>
       </c>
       <c r="F96" t="s">
-        <v>292</v>
+        <v>250</v>
       </c>
       <c r="G96" t="b">
         <v>0</v>
       </c>
       <c r="H96" t="s">
-        <v>663</v>
+        <v>628</v>
       </c>
       <c r="I96" t="s">
-        <v>399</v>
+        <v>678</v>
       </c>
       <c r="J96" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="K96" t="s">
         <v>687</v>
       </c>
       <c r="L96" t="s">
-        <v>710</v>
+        <v>698</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="B97" t="s">
-        <v>523</v>
+        <v>484</v>
       </c>
       <c r="C97">
-        <v>-200000</v>
+        <v>26</v>
       </c>
       <c r="D97" t="s">
-        <v>596</v>
+        <v>589</v>
       </c>
       <c r="E97">
         <v>1</v>
       </c>
       <c r="F97" t="s">
-        <v>292</v>
+        <v>251</v>
       </c>
       <c r="G97" t="b">
         <v>0</v>
       </c>
       <c r="H97" t="s">
-        <v>662</v>
+        <v>626</v>
       </c>
       <c r="I97" t="s">
-        <v>398</v>
+        <v>678</v>
       </c>
       <c r="J97" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="K97" t="s">
         <v>687</v>
       </c>
       <c r="L97" t="s">
-        <v>710</v>
+        <v>698</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="B98" t="s">
-        <v>456</v>
+        <v>514</v>
       </c>
       <c r="C98">
-        <v>-1161035</v>
+        <v>-1000000</v>
       </c>
       <c r="D98" t="s">
-        <v>584</v>
+        <v>349</v>
       </c>
       <c r="E98">
         <v>1</v>
       </c>
       <c r="F98" t="s">
-        <v>223</v>
+        <v>268</v>
       </c>
       <c r="G98" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H98" t="s">
-        <v>605</v>
+        <v>349</v>
       </c>
       <c r="I98" t="s">
-        <v>676</v>
+        <v>393</v>
       </c>
       <c r="J98" t="s">
         <v>350</v>
       </c>
       <c r="K98" t="s">
+        <v>686</v>
+      </c>
+      <c r="L98" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A99" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="C99" s="3">
+        <v>-500</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E99" s="3">
+        <v>1</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="G99" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="J99" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K99" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L98" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>15</v>
-      </c>
-      <c r="B99" t="s">
-        <v>454</v>
-      </c>
-      <c r="C99">
-        <v>-8471713</v>
-      </c>
-      <c r="D99" t="s">
-        <v>584</v>
-      </c>
-      <c r="E99">
-        <v>1</v>
-      </c>
-      <c r="F99" t="s">
-        <v>221</v>
-      </c>
-      <c r="G99" t="b">
-        <v>0</v>
-      </c>
-      <c r="H99" t="s">
-        <v>603</v>
-      </c>
-      <c r="I99" t="s">
-        <v>676</v>
-      </c>
-      <c r="J99" t="s">
-        <v>350</v>
-      </c>
-      <c r="K99" t="s">
-        <v>687</v>
-      </c>
-      <c r="L99" t="s">
-        <v>692</v>
+      <c r="L99" s="3" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>455</v>
+        <v>523</v>
       </c>
       <c r="C100">
-        <v>-1161035</v>
+        <v>-60000</v>
       </c>
       <c r="D100" t="s">
-        <v>584</v>
+        <v>596</v>
       </c>
       <c r="E100">
         <v>1</v>
       </c>
       <c r="F100" t="s">
-        <v>222</v>
+        <v>292</v>
       </c>
       <c r="G100" t="b">
         <v>0</v>
       </c>
       <c r="H100" t="s">
-        <v>604</v>
+        <v>663</v>
       </c>
       <c r="I100" t="s">
-        <v>676</v>
+        <v>399</v>
       </c>
       <c r="J100" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="K100" t="s">
         <v>687</v>
       </c>
       <c r="L100" t="s">
-        <v>692</v>
+        <v>710</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B101" t="s">
-        <v>456</v>
+        <v>523</v>
       </c>
       <c r="C101">
-        <v>-5712018</v>
+        <v>-200000</v>
       </c>
       <c r="D101" t="s">
-        <v>584</v>
+        <v>596</v>
       </c>
       <c r="E101">
         <v>1</v>
       </c>
       <c r="F101" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="G101" t="b">
         <v>0</v>
       </c>
       <c r="H101" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="I101" t="s">
-        <v>682</v>
+        <v>398</v>
       </c>
       <c r="J101" t="s">
         <v>350</v>
@@ -20692,18 +20778,18 @@
         <v>687</v>
       </c>
       <c r="L101" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="B102" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C102">
-        <v>-4656642</v>
+        <v>-1161035</v>
       </c>
       <c r="D102" t="s">
         <v>584</v>
@@ -20712,16 +20798,16 @@
         <v>1</v>
       </c>
       <c r="F102" t="s">
-        <v>282</v>
+        <v>223</v>
       </c>
       <c r="G102" t="b">
         <v>0</v>
       </c>
       <c r="H102" t="s">
-        <v>657</v>
+        <v>605</v>
       </c>
       <c r="I102" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="J102" t="s">
         <v>350</v>
@@ -20730,18 +20816,18 @@
         <v>687</v>
       </c>
       <c r="L102" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>91</v>
+        <v>15</v>
       </c>
       <c r="B103" t="s">
-        <v>522</v>
+        <v>454</v>
       </c>
       <c r="C103">
-        <v>-1428005</v>
+        <v>-8471713</v>
       </c>
       <c r="D103" t="s">
         <v>584</v>
@@ -20750,16 +20836,16 @@
         <v>1</v>
       </c>
       <c r="F103" t="s">
-        <v>285</v>
+        <v>221</v>
       </c>
       <c r="G103" t="b">
         <v>0</v>
       </c>
       <c r="H103" t="s">
-        <v>660</v>
+        <v>603</v>
       </c>
       <c r="I103" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="J103" t="s">
         <v>350</v>
@@ -20768,18 +20854,18 @@
         <v>687</v>
       </c>
       <c r="L103" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="B104" t="s">
         <v>455</v>
       </c>
       <c r="C104">
-        <v>-5712018</v>
+        <v>-1161035</v>
       </c>
       <c r="D104" t="s">
         <v>584</v>
@@ -20788,16 +20874,16 @@
         <v>1</v>
       </c>
       <c r="F104" t="s">
-        <v>283</v>
+        <v>222</v>
       </c>
       <c r="G104" t="b">
         <v>0</v>
       </c>
       <c r="H104" t="s">
-        <v>658</v>
+        <v>604</v>
       </c>
       <c r="I104" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="J104" t="s">
         <v>350</v>
@@ -20806,18 +20892,18 @@
         <v>687</v>
       </c>
       <c r="L104" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="B105" t="s">
         <v>456</v>
       </c>
       <c r="C105">
-        <v>-9817684</v>
+        <v>-5712018</v>
       </c>
       <c r="D105" t="s">
         <v>584</v>
@@ -20826,16 +20912,16 @@
         <v>1</v>
       </c>
       <c r="F105" t="s">
-        <v>302</v>
+        <v>284</v>
       </c>
       <c r="G105" t="b">
         <v>0</v>
       </c>
       <c r="H105" t="s">
-        <v>669</v>
+        <v>659</v>
       </c>
       <c r="I105" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="J105" t="s">
         <v>350</v>
@@ -20844,18 +20930,18 @@
         <v>687</v>
       </c>
       <c r="L105" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="B106" t="s">
         <v>454</v>
       </c>
       <c r="C106">
-        <v>-4622358</v>
+        <v>-4656642</v>
       </c>
       <c r="D106" t="s">
         <v>584</v>
@@ -20864,7 +20950,7 @@
         <v>1</v>
       </c>
       <c r="F106" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="G106" t="b">
         <v>0</v>
@@ -20873,7 +20959,7 @@
         <v>657</v>
       </c>
       <c r="I106" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="J106" t="s">
         <v>350</v>
@@ -20882,18 +20968,18 @@
         <v>687</v>
       </c>
       <c r="L106" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="B107" t="s">
         <v>522</v>
       </c>
       <c r="C107">
-        <v>-2454421</v>
+        <v>-1428005</v>
       </c>
       <c r="D107" t="s">
         <v>584</v>
@@ -20902,16 +20988,16 @@
         <v>1</v>
       </c>
       <c r="F107" t="s">
-        <v>303</v>
+        <v>285</v>
       </c>
       <c r="G107" t="b">
         <v>0</v>
       </c>
       <c r="H107" t="s">
-        <v>670</v>
+        <v>660</v>
       </c>
       <c r="I107" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="J107" t="s">
         <v>350</v>
@@ -20920,18 +21006,18 @@
         <v>687</v>
       </c>
       <c r="L107" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="B108" t="s">
         <v>455</v>
       </c>
       <c r="C108">
-        <v>-9817684</v>
+        <v>-5712018</v>
       </c>
       <c r="D108" t="s">
         <v>584</v>
@@ -20940,16 +21026,16 @@
         <v>1</v>
       </c>
       <c r="F108" t="s">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="G108" t="b">
         <v>0</v>
       </c>
       <c r="H108" t="s">
-        <v>668</v>
+        <v>658</v>
       </c>
       <c r="I108" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="J108" t="s">
         <v>350</v>
@@ -20958,112 +21044,112 @@
         <v>687</v>
       </c>
       <c r="L108" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="B109" t="s">
-        <v>515</v>
+        <v>456</v>
       </c>
       <c r="C109">
-        <v>-1000000</v>
+        <v>-9817684</v>
       </c>
       <c r="D109" t="s">
-        <v>349</v>
+        <v>584</v>
       </c>
       <c r="E109">
         <v>1</v>
       </c>
       <c r="F109" t="s">
-        <v>270</v>
+        <v>302</v>
       </c>
       <c r="G109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H109" t="s">
-        <v>349</v>
+        <v>669</v>
       </c>
       <c r="I109" t="s">
-        <v>393</v>
+        <v>684</v>
       </c>
       <c r="J109" t="s">
         <v>350</v>
       </c>
       <c r="K109" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L109" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A110" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B110" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="C110" s="3">
-        <v>-500</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="E110" s="3">
-        <v>1</v>
-      </c>
-      <c r="F110" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="G110" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H110" s="3" t="s">
-        <v>641</v>
-      </c>
-      <c r="I110" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="J110" s="3" t="s">
+      <c r="A110" t="s">
+        <v>107</v>
+      </c>
+      <c r="B110" t="s">
+        <v>454</v>
+      </c>
+      <c r="C110">
+        <v>-4622358</v>
+      </c>
+      <c r="D110" t="s">
+        <v>584</v>
+      </c>
+      <c r="E110">
+        <v>1</v>
+      </c>
+      <c r="F110" t="s">
+        <v>300</v>
+      </c>
+      <c r="G110" t="b">
+        <v>0</v>
+      </c>
+      <c r="H110" t="s">
+        <v>657</v>
+      </c>
+      <c r="I110" t="s">
+        <v>684</v>
+      </c>
+      <c r="J110" t="s">
         <v>350</v>
       </c>
-      <c r="K110" s="3" t="s">
+      <c r="K110" t="s">
         <v>687</v>
       </c>
-      <c r="L110" s="3" t="s">
-        <v>700</v>
+      <c r="L110" t="s">
+        <v>713</v>
       </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>459</v>
+        <v>522</v>
       </c>
       <c r="C111">
-        <v>-410000</v>
+        <v>-2454421</v>
       </c>
       <c r="D111" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E111">
         <v>1</v>
       </c>
       <c r="F111" t="s">
-        <v>226</v>
+        <v>303</v>
       </c>
       <c r="G111" t="b">
         <v>0</v>
       </c>
       <c r="H111" t="s">
-        <v>608</v>
+        <v>670</v>
       </c>
       <c r="I111" t="s">
-        <v>384</v>
+        <v>684</v>
       </c>
       <c r="J111" t="s">
         <v>350</v>
@@ -21072,36 +21158,36 @@
         <v>687</v>
       </c>
       <c r="L111" t="s">
-        <v>694</v>
+        <v>713</v>
       </c>
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>21</v>
+        <v>108</v>
       </c>
       <c r="B112" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="C112">
-        <v>-14000</v>
+        <v>-9817684</v>
       </c>
       <c r="D112" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E112">
         <v>1</v>
       </c>
       <c r="F112" t="s">
-        <v>227</v>
+        <v>301</v>
       </c>
       <c r="G112" t="b">
         <v>0</v>
       </c>
       <c r="H112" t="s">
-        <v>609</v>
+        <v>668</v>
       </c>
       <c r="I112" t="s">
-        <v>384</v>
+        <v>684</v>
       </c>
       <c r="J112" t="s">
         <v>350</v>
@@ -21110,112 +21196,112 @@
         <v>687</v>
       </c>
       <c r="L112" t="s">
-        <v>694</v>
+        <v>713</v>
       </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="B113" t="s">
-        <v>461</v>
+        <v>515</v>
       </c>
       <c r="C113">
-        <v>-53000</v>
+        <v>-1000000</v>
       </c>
       <c r="D113" t="s">
-        <v>586</v>
+        <v>349</v>
       </c>
       <c r="E113">
         <v>1</v>
       </c>
       <c r="F113" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="G113" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H113" t="s">
-        <v>610</v>
+        <v>349</v>
       </c>
       <c r="I113" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
       <c r="J113" t="s">
         <v>350</v>
       </c>
       <c r="K113" t="s">
+        <v>686</v>
+      </c>
+      <c r="L113" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A114" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="C114" s="3">
+        <v>-500</v>
+      </c>
+      <c r="D114" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E114" s="3">
+        <v>1</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G114" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="I114" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="J114" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K114" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L113" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>23</v>
-      </c>
-      <c r="B114" t="s">
-        <v>462</v>
-      </c>
-      <c r="C114">
-        <v>-10000</v>
-      </c>
-      <c r="D114" t="s">
-        <v>586</v>
-      </c>
-      <c r="E114">
-        <v>1</v>
-      </c>
-      <c r="F114" t="s">
-        <v>229</v>
-      </c>
-      <c r="G114" t="b">
-        <v>0</v>
-      </c>
-      <c r="H114" t="s">
-        <v>611</v>
-      </c>
-      <c r="I114" t="s">
-        <v>384</v>
-      </c>
-      <c r="J114" t="s">
-        <v>349</v>
-      </c>
-      <c r="K114" t="s">
-        <v>687</v>
-      </c>
-      <c r="L114" t="s">
-        <v>694</v>
+      <c r="L114" s="3" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="B115" t="s">
-        <v>505</v>
+        <v>459</v>
       </c>
       <c r="C115">
-        <v>-0.06</v>
+        <v>-410000</v>
       </c>
       <c r="D115" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="E115">
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>272</v>
+        <v>226</v>
       </c>
       <c r="G115" t="b">
         <v>0</v>
       </c>
       <c r="H115" t="s">
-        <v>643</v>
+        <v>608</v>
       </c>
       <c r="I115" t="s">
-        <v>680</v>
+        <v>384</v>
       </c>
       <c r="J115" t="s">
         <v>350</v>
@@ -21224,36 +21310,36 @@
         <v>687</v>
       </c>
       <c r="L115" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="B116" t="s">
-        <v>506</v>
+        <v>460</v>
       </c>
       <c r="C116">
-        <v>-1.7000000000000001E-2</v>
+        <v>-14000</v>
       </c>
       <c r="D116" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="E116">
         <v>1</v>
       </c>
       <c r="F116" t="s">
-        <v>273</v>
+        <v>227</v>
       </c>
       <c r="G116" t="b">
         <v>0</v>
       </c>
       <c r="H116" t="s">
-        <v>644</v>
+        <v>609</v>
       </c>
       <c r="I116" t="s">
-        <v>680</v>
+        <v>384</v>
       </c>
       <c r="J116" t="s">
         <v>350</v>
@@ -21262,399 +21348,399 @@
         <v>687</v>
       </c>
       <c r="L116" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A117" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="C117" s="3">
-        <v>-0.48</v>
-      </c>
-      <c r="D117" s="3" t="s">
-        <v>594</v>
-      </c>
-      <c r="E117" s="3">
-        <v>1</v>
-      </c>
-      <c r="F117" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="G117" s="3" t="b">
+      <c r="A117" t="s">
+        <v>22</v>
+      </c>
+      <c r="B117" t="s">
+        <v>461</v>
+      </c>
+      <c r="C117">
+        <v>-53000</v>
+      </c>
+      <c r="D117" t="s">
+        <v>586</v>
+      </c>
+      <c r="E117">
+        <v>1</v>
+      </c>
+      <c r="F117" t="s">
+        <v>228</v>
+      </c>
+      <c r="G117" t="b">
         <v>0</v>
       </c>
-      <c r="H117" s="3" t="s">
-        <v>645</v>
-      </c>
-      <c r="I117" s="3" t="s">
-        <v>680</v>
-      </c>
-      <c r="J117" s="3" t="s">
+      <c r="H117" t="s">
+        <v>610</v>
+      </c>
+      <c r="I117" t="s">
+        <v>384</v>
+      </c>
+      <c r="J117" t="s">
         <v>350</v>
       </c>
-      <c r="K117" s="3" t="s">
+      <c r="K117" t="s">
         <v>687</v>
       </c>
-      <c r="L117" s="3" t="s">
-        <v>702</v>
+      <c r="L117" t="s">
+        <v>694</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="B118" t="s">
-        <v>508</v>
+        <v>462</v>
       </c>
       <c r="C118">
-        <v>-14</v>
+        <v>-10000</v>
       </c>
       <c r="D118" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="E118">
         <v>1</v>
       </c>
       <c r="F118" t="s">
-        <v>275</v>
+        <v>229</v>
       </c>
       <c r="G118" t="b">
         <v>0</v>
       </c>
       <c r="H118" t="s">
-        <v>646</v>
+        <v>611</v>
       </c>
       <c r="I118" t="s">
-        <v>680</v>
+        <v>384</v>
       </c>
       <c r="J118" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="K118" t="s">
         <v>687</v>
       </c>
       <c r="L118" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>67</v>
+      </c>
+      <c r="B119" t="s">
+        <v>505</v>
+      </c>
+      <c r="C119">
+        <v>-0.06</v>
+      </c>
+      <c r="D119" t="s">
+        <v>593</v>
+      </c>
+      <c r="E119">
+        <v>1</v>
+      </c>
+      <c r="F119" t="s">
+        <v>272</v>
+      </c>
+      <c r="G119" t="b">
+        <v>0</v>
+      </c>
+      <c r="H119" t="s">
+        <v>643</v>
+      </c>
+      <c r="I119" t="s">
+        <v>680</v>
+      </c>
+      <c r="J119" t="s">
+        <v>350</v>
+      </c>
+      <c r="K119" t="s">
+        <v>687</v>
+      </c>
+      <c r="L119" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A119" s="3" t="s">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>68</v>
+      </c>
+      <c r="B120" t="s">
+        <v>506</v>
+      </c>
+      <c r="C120">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+      <c r="D120" t="s">
+        <v>594</v>
+      </c>
+      <c r="E120">
+        <v>1</v>
+      </c>
+      <c r="F120" t="s">
+        <v>273</v>
+      </c>
+      <c r="G120" t="b">
+        <v>0</v>
+      </c>
+      <c r="H120" t="s">
+        <v>644</v>
+      </c>
+      <c r="I120" t="s">
+        <v>680</v>
+      </c>
+      <c r="J120" t="s">
+        <v>350</v>
+      </c>
+      <c r="K120" t="s">
+        <v>687</v>
+      </c>
+      <c r="L120" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A121" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="C121" s="3">
+        <v>-0.48</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="E121" s="3">
+        <v>1</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G121" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H121" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="I121" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="J121" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="K121" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="L121" s="3" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>70</v>
+      </c>
+      <c r="B122" t="s">
+        <v>508</v>
+      </c>
+      <c r="C122">
+        <v>-14</v>
+      </c>
+      <c r="D122" t="s">
+        <v>594</v>
+      </c>
+      <c r="E122">
+        <v>1</v>
+      </c>
+      <c r="F122" t="s">
+        <v>275</v>
+      </c>
+      <c r="G122" t="b">
+        <v>0</v>
+      </c>
+      <c r="H122" t="s">
+        <v>646</v>
+      </c>
+      <c r="I122" t="s">
+        <v>680</v>
+      </c>
+      <c r="J122" t="s">
+        <v>350</v>
+      </c>
+      <c r="K122" t="s">
+        <v>687</v>
+      </c>
+      <c r="L122" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A123" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B119" s="3" t="s">
+      <c r="B123" s="3" t="s">
         <v>509</v>
       </c>
-      <c r="C119" s="3">
+      <c r="C123" s="3">
         <v>-0.05</v>
       </c>
-      <c r="D119" s="3" t="s">
+      <c r="D123" s="3" t="s">
         <v>594</v>
       </c>
-      <c r="E119" s="3">
-        <v>1</v>
-      </c>
-      <c r="F119" s="3" t="s">
+      <c r="E123" s="3">
+        <v>1</v>
+      </c>
+      <c r="F123" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="G119" s="3" t="b">
+      <c r="G123" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H119" s="3" t="s">
+      <c r="H123" s="3" t="s">
         <v>647</v>
       </c>
-      <c r="I119" s="3" t="s">
+      <c r="I123" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="J119" s="3" t="s">
+      <c r="J123" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="K119" s="3" t="s">
+      <c r="K123" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L119" s="3" t="s">
+      <c r="L123" s="3" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A120" s="3" t="s">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A124" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B120" s="3" t="s">
+      <c r="B124" s="3" t="s">
         <v>510</v>
       </c>
-      <c r="C120" s="3">
+      <c r="C124" s="3">
         <f>-0.1/10</f>
         <v>-0.01</v>
       </c>
-      <c r="D120" s="3" t="s">
+      <c r="D124" s="3" t="s">
         <v>594</v>
       </c>
-      <c r="E120" s="3">
-        <v>1</v>
-      </c>
-      <c r="F120" s="3" t="s">
+      <c r="E124" s="3">
+        <v>1</v>
+      </c>
+      <c r="F124" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="G120" s="3" t="b">
+      <c r="G124" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="H120" s="3" t="s">
+      <c r="H124" s="3" t="s">
         <v>648</v>
       </c>
-      <c r="I120" s="3" t="s">
+      <c r="I124" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="J120" s="3" t="s">
+      <c r="J124" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="K120" s="3" t="s">
+      <c r="K124" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="L120" s="3" t="s">
+      <c r="L124" s="3" t="s">
         <v>702</v>
-      </c>
-    </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
-        <v>60</v>
-      </c>
-      <c r="B121" t="s">
-        <v>498</v>
-      </c>
-      <c r="C121">
-        <v>323.52941179999999</v>
-      </c>
-      <c r="D121" t="s">
-        <v>591</v>
-      </c>
-      <c r="E121">
-        <v>1</v>
-      </c>
-      <c r="F121" t="s">
-        <v>265</v>
-      </c>
-      <c r="G121" t="b">
-        <v>1</v>
-      </c>
-      <c r="H121" t="s">
-        <v>640</v>
-      </c>
-      <c r="I121" t="s">
-        <v>349</v>
-      </c>
-      <c r="J121" t="s">
-        <v>354</v>
-      </c>
-      <c r="K121" t="s">
-        <v>687</v>
-      </c>
-      <c r="L121" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>59</v>
-      </c>
-      <c r="B122" t="s">
-        <v>498</v>
-      </c>
-      <c r="C122">
-        <v>-500</v>
-      </c>
-      <c r="D122" t="s">
-        <v>591</v>
-      </c>
-      <c r="E122">
-        <v>1</v>
-      </c>
-      <c r="F122" t="s">
-        <v>265</v>
-      </c>
-      <c r="G122" t="b">
-        <v>1</v>
-      </c>
-      <c r="H122" t="s">
-        <v>639</v>
-      </c>
-      <c r="I122" t="s">
-        <v>349</v>
-      </c>
-      <c r="J122" t="s">
-        <v>353</v>
-      </c>
-      <c r="K122" t="s">
-        <v>687</v>
-      </c>
-      <c r="L122" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
-        <v>32</v>
-      </c>
-      <c r="B123" t="s">
-        <v>471</v>
-      </c>
-      <c r="C123">
-        <v>-0.64</v>
-      </c>
-      <c r="D123" t="s">
-        <v>588</v>
-      </c>
-      <c r="E123">
-        <v>1</v>
-      </c>
-      <c r="F123" t="s">
-        <v>238</v>
-      </c>
-      <c r="G123" t="b">
-        <v>0</v>
-      </c>
-      <c r="H123" t="s">
-        <v>620</v>
-      </c>
-      <c r="I123" t="s">
-        <v>386</v>
-      </c>
-      <c r="J123" t="s">
-        <v>351</v>
-      </c>
-      <c r="K123" t="s">
-        <v>687</v>
-      </c>
-      <c r="L123" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
-        <v>33</v>
-      </c>
-      <c r="B124" t="s">
-        <v>472</v>
-      </c>
-      <c r="C124">
-        <v>-1.44</v>
-      </c>
-      <c r="D124" t="s">
-        <v>588</v>
-      </c>
-      <c r="E124">
-        <v>1</v>
-      </c>
-      <c r="F124" t="s">
-        <v>239</v>
-      </c>
-      <c r="G124" t="b">
-        <v>0</v>
-      </c>
-      <c r="H124" t="s">
-        <v>621</v>
-      </c>
-      <c r="I124" t="s">
-        <v>386</v>
-      </c>
-      <c r="J124" t="s">
-        <v>351</v>
-      </c>
-      <c r="K124" t="s">
-        <v>687</v>
-      </c>
-      <c r="L124" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="B125" t="s">
-        <v>473</v>
+        <v>498</v>
       </c>
       <c r="C125">
-        <v>-1.44</v>
+        <v>323.52941179999999</v>
       </c>
       <c r="D125" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E125">
         <v>1</v>
       </c>
       <c r="F125" t="s">
-        <v>240</v>
+        <v>265</v>
       </c>
       <c r="G125" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H125" t="s">
-        <v>621</v>
+        <v>640</v>
       </c>
       <c r="I125" t="s">
-        <v>386</v>
+        <v>349</v>
       </c>
       <c r="J125" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="K125" t="s">
         <v>687</v>
       </c>
       <c r="L125" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="B126" t="s">
-        <v>469</v>
+        <v>498</v>
       </c>
       <c r="C126">
-        <v>-3.04</v>
+        <v>-500</v>
       </c>
       <c r="D126" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E126">
         <v>1</v>
       </c>
       <c r="F126" t="s">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="G126" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H126" t="s">
-        <v>618</v>
+        <v>639</v>
       </c>
       <c r="I126" t="s">
-        <v>386</v>
+        <v>349</v>
       </c>
       <c r="J126" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="K126" t="s">
         <v>687</v>
       </c>
       <c r="L126" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B127" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C127">
-        <v>-3.04</v>
+        <v>-0.64</v>
       </c>
       <c r="D127" t="s">
         <v>588</v>
@@ -21663,13 +21749,13 @@
         <v>1</v>
       </c>
       <c r="F127" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G127" t="b">
         <v>0</v>
       </c>
       <c r="H127" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="I127" t="s">
         <v>386</v>
@@ -21686,13 +21772,13 @@
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B128" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C128">
-        <v>-0.06</v>
+        <v>-1.44</v>
       </c>
       <c r="D128" t="s">
         <v>588</v>
@@ -21701,13 +21787,13 @@
         <v>1</v>
       </c>
       <c r="F128" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G128" t="b">
         <v>0</v>
       </c>
       <c r="H128" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="I128" t="s">
         <v>386</v>
@@ -21724,317 +21810,317 @@
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="B129" t="s">
-        <v>534</v>
+        <v>473</v>
       </c>
       <c r="C129">
-        <v>60</v>
+        <v>-1.44</v>
       </c>
       <c r="D129" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E129">
         <v>1</v>
       </c>
       <c r="F129" t="s">
-        <v>307</v>
+        <v>240</v>
       </c>
       <c r="G129" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H129" t="s">
-        <v>674</v>
+        <v>621</v>
       </c>
       <c r="I129" t="s">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="J129" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K129" t="s">
         <v>687</v>
       </c>
       <c r="L129" t="s">
-        <v>714</v>
+        <v>696</v>
       </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>113</v>
+        <v>30</v>
       </c>
       <c r="B130" t="s">
-        <v>533</v>
+        <v>469</v>
       </c>
       <c r="C130">
-        <v>130</v>
+        <v>-3.04</v>
       </c>
       <c r="D130" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E130">
         <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>306</v>
+        <v>236</v>
       </c>
       <c r="G130" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H130" t="s">
-        <v>673</v>
+        <v>618</v>
       </c>
       <c r="I130" t="s">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="J130" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K130" t="s">
         <v>687</v>
       </c>
       <c r="L130" t="s">
-        <v>714</v>
+        <v>696</v>
       </c>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>112</v>
+        <v>31</v>
       </c>
       <c r="B131" t="s">
-        <v>532</v>
+        <v>470</v>
       </c>
       <c r="C131">
-        <v>20000</v>
+        <v>-3.04</v>
       </c>
       <c r="D131" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E131">
         <v>1</v>
       </c>
       <c r="F131" t="s">
-        <v>305</v>
+        <v>237</v>
       </c>
       <c r="G131" t="b">
         <v>0</v>
       </c>
       <c r="H131" t="s">
-        <v>672</v>
+        <v>619</v>
       </c>
       <c r="I131" t="s">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="J131" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K131" t="s">
         <v>687</v>
       </c>
       <c r="L131" t="s">
-        <v>714</v>
+        <v>696</v>
       </c>
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>111</v>
+        <v>35</v>
       </c>
       <c r="B132" t="s">
-        <v>531</v>
+        <v>474</v>
       </c>
       <c r="C132">
-        <v>51000</v>
+        <v>-0.06</v>
       </c>
       <c r="D132" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E132">
         <v>1</v>
       </c>
       <c r="F132" t="s">
-        <v>304</v>
+        <v>241</v>
       </c>
       <c r="G132" t="b">
         <v>0</v>
       </c>
       <c r="H132" t="s">
-        <v>671</v>
+        <v>622</v>
       </c>
       <c r="I132" t="s">
-        <v>685</v>
+        <v>386</v>
       </c>
       <c r="J132" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K132" t="s">
         <v>687</v>
       </c>
       <c r="L132" t="s">
-        <v>714</v>
+        <v>696</v>
       </c>
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>36</v>
+        <v>114</v>
       </c>
       <c r="B133" t="s">
-        <v>475</v>
+        <v>534</v>
       </c>
       <c r="C133">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="D133" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="E133">
         <v>1</v>
       </c>
       <c r="F133" t="s">
-        <v>242</v>
+        <v>307</v>
       </c>
       <c r="G133" t="b">
         <v>1</v>
       </c>
       <c r="H133" t="s">
-        <v>623</v>
+        <v>674</v>
       </c>
       <c r="I133" t="s">
-        <v>387</v>
+        <v>685</v>
       </c>
       <c r="J133" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K133" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L133" t="s">
-        <v>697</v>
+        <v>714</v>
       </c>
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>6</v>
+        <v>113</v>
       </c>
       <c r="B134" t="s">
-        <v>444</v>
+        <v>533</v>
       </c>
       <c r="C134">
-        <v>-68.099999999999994</v>
+        <v>130</v>
       </c>
       <c r="D134" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="E134">
         <v>1</v>
       </c>
       <c r="F134" t="s">
-        <v>211</v>
+        <v>306</v>
       </c>
       <c r="G134" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H134" t="s">
-        <v>598</v>
+        <v>673</v>
       </c>
       <c r="I134" t="s">
-        <v>377</v>
+        <v>685</v>
       </c>
       <c r="J134" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K134" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L134" t="s">
-        <v>689</v>
+        <v>714</v>
       </c>
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>9</v>
+        <v>112</v>
       </c>
       <c r="B135" t="s">
-        <v>447</v>
+        <v>532</v>
       </c>
       <c r="C135">
-        <v>-34.1</v>
+        <v>20000</v>
       </c>
       <c r="D135" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="E135">
         <v>1</v>
       </c>
       <c r="F135" t="s">
-        <v>214</v>
+        <v>305</v>
       </c>
       <c r="G135" t="b">
         <v>0</v>
       </c>
       <c r="H135" t="s">
-        <v>600</v>
+        <v>672</v>
       </c>
       <c r="I135" t="s">
-        <v>377</v>
+        <v>685</v>
       </c>
       <c r="J135" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K135" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L135" t="s">
-        <v>689</v>
+        <v>714</v>
       </c>
     </row>
     <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="B136" t="s">
-        <v>449</v>
+        <v>531</v>
       </c>
       <c r="C136">
-        <v>0</v>
+        <v>51000</v>
       </c>
       <c r="D136" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="E136">
         <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>216</v>
+        <v>304</v>
       </c>
       <c r="G136" t="b">
         <v>0</v>
       </c>
       <c r="H136" t="s">
-        <v>349</v>
+        <v>671</v>
       </c>
       <c r="I136" t="s">
-        <v>378</v>
+        <v>685</v>
       </c>
       <c r="J136" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K136" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="L136" t="s">
-        <v>689</v>
+        <v>714</v>
       </c>
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="B137" t="s">
-        <v>445</v>
+        <v>475</v>
       </c>
       <c r="C137">
-        <v>-102.1</v>
+        <v>200</v>
       </c>
       <c r="D137" t="s">
         <v>583</v>
@@ -22043,16 +22129,16 @@
         <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="G137" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H137" t="s">
-        <v>599</v>
+        <v>623</v>
       </c>
       <c r="I137" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="J137" t="s">
         <v>349</v>
@@ -22061,18 +22147,18 @@
         <v>686</v>
       </c>
       <c r="L137" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B138" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="C138">
-        <v>-66.2</v>
+        <v>-68.099999999999994</v>
       </c>
       <c r="D138" t="s">
         <v>583</v>
@@ -22081,13 +22167,13 @@
         <v>1</v>
       </c>
       <c r="F138" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G138" t="b">
         <v>0</v>
       </c>
       <c r="H138" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="I138" t="s">
         <v>377</v>
@@ -22104,13 +22190,13 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B139" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="C139">
-        <v>-6.5</v>
+        <v>-34.1</v>
       </c>
       <c r="D139" t="s">
         <v>583</v>
@@ -22119,13 +22205,13 @@
         <v>1</v>
       </c>
       <c r="F139" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="G139" t="b">
         <v>0</v>
       </c>
       <c r="H139" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="I139" t="s">
         <v>377</v>
@@ -22142,13 +22228,13 @@
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B140" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="C140">
-        <v>-6.5</v>
+        <v>0</v>
       </c>
       <c r="D140" t="s">
         <v>583</v>
@@ -22157,16 +22243,16 @@
         <v>1</v>
       </c>
       <c r="F140" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G140" t="b">
         <v>0</v>
       </c>
       <c r="H140" t="s">
-        <v>597</v>
+        <v>349</v>
       </c>
       <c r="I140" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J140" t="s">
         <v>349</v>
@@ -22180,183 +22266,183 @@
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="B141" t="s">
-        <v>467</v>
+        <v>445</v>
       </c>
       <c r="C141">
-        <v>-115</v>
+        <v>-102.1</v>
       </c>
       <c r="D141" t="s">
-        <v>590</v>
+        <v>583</v>
       </c>
       <c r="E141">
         <v>1</v>
       </c>
       <c r="F141" t="s">
-        <v>278</v>
+        <v>212</v>
       </c>
       <c r="G141" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H141" t="s">
-        <v>649</v>
+        <v>599</v>
       </c>
       <c r="I141" t="s">
-        <v>392</v>
+        <v>377</v>
       </c>
       <c r="J141" t="s">
         <v>349</v>
       </c>
       <c r="K141" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="L141" t="s">
-        <v>703</v>
+        <v>689</v>
       </c>
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="B142" t="s">
-        <v>517</v>
+        <v>448</v>
       </c>
       <c r="C142">
-        <v>323.52941179999999</v>
+        <v>-66.2</v>
       </c>
       <c r="D142" t="s">
-        <v>595</v>
+        <v>583</v>
       </c>
       <c r="E142">
         <v>1</v>
       </c>
       <c r="F142" t="s">
-        <v>280</v>
+        <v>215</v>
       </c>
       <c r="G142" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H142" t="s">
-        <v>653</v>
+        <v>601</v>
       </c>
       <c r="I142" t="s">
-        <v>394</v>
+        <v>377</v>
       </c>
       <c r="J142" t="s">
         <v>349</v>
       </c>
       <c r="K142" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="L142" t="s">
-        <v>706</v>
+        <v>689</v>
       </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>84</v>
+        <v>5</v>
       </c>
       <c r="B143" t="s">
-        <v>518</v>
+        <v>443</v>
       </c>
       <c r="C143">
-        <v>323.52941179999999</v>
+        <v>-6.5</v>
       </c>
       <c r="D143" t="s">
-        <v>595</v>
+        <v>583</v>
       </c>
       <c r="E143">
         <v>1</v>
       </c>
       <c r="F143" t="s">
-        <v>281</v>
+        <v>210</v>
       </c>
       <c r="G143" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H143" t="s">
-        <v>653</v>
+        <v>597</v>
       </c>
       <c r="I143" t="s">
-        <v>394</v>
+        <v>377</v>
       </c>
       <c r="J143" t="s">
         <v>349</v>
       </c>
       <c r="K143" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="L143" t="s">
-        <v>706</v>
+        <v>689</v>
       </c>
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="B144" t="s">
-        <v>463</v>
+        <v>446</v>
       </c>
       <c r="C144">
-        <v>-86</v>
+        <v>-6.5</v>
       </c>
       <c r="D144" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E144">
         <v>1</v>
       </c>
       <c r="F144" t="s">
-        <v>286</v>
+        <v>213</v>
       </c>
       <c r="G144" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H144" t="s">
-        <v>661</v>
+        <v>597</v>
       </c>
       <c r="I144" t="s">
-        <v>397</v>
+        <v>377</v>
       </c>
       <c r="J144" t="s">
         <v>349</v>
       </c>
       <c r="K144" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="L144" t="s">
-        <v>709</v>
+        <v>689</v>
       </c>
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="B145" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="C145">
-        <v>-86</v>
+        <v>-115</v>
       </c>
       <c r="D145" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="E145">
         <v>1</v>
       </c>
       <c r="F145" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="G145" t="b">
         <v>1</v>
       </c>
       <c r="H145" t="s">
-        <v>661</v>
+        <v>649</v>
       </c>
       <c r="I145" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="J145" t="s">
         <v>349</v>
@@ -22365,36 +22451,36 @@
         <v>687</v>
       </c>
       <c r="L145" t="s">
-        <v>709</v>
+        <v>703</v>
       </c>
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B146" t="s">
-        <v>465</v>
+        <v>517</v>
       </c>
       <c r="C146">
-        <v>-86</v>
+        <v>323.52941179999999</v>
       </c>
       <c r="D146" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="E146">
         <v>1</v>
       </c>
       <c r="F146" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="G146" t="b">
         <v>1</v>
       </c>
       <c r="H146" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
       <c r="I146" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="J146" t="s">
         <v>349</v>
@@ -22403,36 +22489,36 @@
         <v>687</v>
       </c>
       <c r="L146" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B147" t="s">
-        <v>466</v>
+        <v>518</v>
       </c>
       <c r="C147">
-        <v>-86</v>
+        <v>323.52941179999999</v>
       </c>
       <c r="D147" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="E147">
         <v>1</v>
       </c>
       <c r="F147" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="G147" t="b">
         <v>1</v>
       </c>
       <c r="H147" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
       <c r="I147" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="J147" t="s">
         <v>349</v>
@@ -22441,18 +22527,18 @@
         <v>687</v>
       </c>
       <c r="L147" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B148" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="C148">
-        <v>-60.2</v>
+        <v>-86</v>
       </c>
       <c r="D148" t="s">
         <v>587</v>
@@ -22461,7 +22547,7 @@
         <v>1</v>
       </c>
       <c r="F148" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="G148" t="b">
         <v>1</v>
@@ -22484,13 +22570,13 @@
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B149" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C149">
-        <v>-60.2</v>
+        <v>-86</v>
       </c>
       <c r="D149" t="s">
         <v>587</v>
@@ -22499,7 +22585,7 @@
         <v>1</v>
       </c>
       <c r="F149" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="G149" t="b">
         <v>1</v>
@@ -22522,10 +22608,10 @@
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="B150" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C150">
         <v>-86</v>
@@ -22537,16 +22623,16 @@
         <v>1</v>
       </c>
       <c r="F150" t="s">
-        <v>230</v>
+        <v>288</v>
       </c>
       <c r="G150" t="b">
         <v>1</v>
       </c>
       <c r="H150" t="s">
-        <v>612</v>
+        <v>661</v>
       </c>
       <c r="I150" t="s">
-        <v>677</v>
+        <v>397</v>
       </c>
       <c r="J150" t="s">
         <v>349</v>
@@ -22555,18 +22641,18 @@
         <v>687</v>
       </c>
       <c r="L150" t="s">
-        <v>695</v>
+        <v>709</v>
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="B151" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C151">
-        <v>-61</v>
+        <v>-86</v>
       </c>
       <c r="D151" t="s">
         <v>587</v>
@@ -22575,16 +22661,16 @@
         <v>1</v>
       </c>
       <c r="F151" t="s">
-        <v>231</v>
+        <v>289</v>
       </c>
       <c r="G151" t="b">
         <v>1</v>
       </c>
       <c r="H151" t="s">
-        <v>613</v>
+        <v>661</v>
       </c>
       <c r="I151" t="s">
-        <v>677</v>
+        <v>397</v>
       </c>
       <c r="J151" t="s">
         <v>349</v>
@@ -22593,18 +22679,18 @@
         <v>687</v>
       </c>
       <c r="L151" t="s">
-        <v>695</v>
+        <v>709</v>
       </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>26</v>
+        <v>96</v>
       </c>
       <c r="B152" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C152">
-        <v>-70</v>
+        <v>-60.2</v>
       </c>
       <c r="D152" t="s">
         <v>587</v>
@@ -22613,16 +22699,16 @@
         <v>1</v>
       </c>
       <c r="F152" t="s">
-        <v>232</v>
+        <v>290</v>
       </c>
       <c r="G152" t="b">
         <v>1</v>
       </c>
       <c r="H152" t="s">
-        <v>614</v>
+        <v>661</v>
       </c>
       <c r="I152" t="s">
-        <v>677</v>
+        <v>397</v>
       </c>
       <c r="J152" t="s">
         <v>349</v>
@@ -22631,18 +22717,18 @@
         <v>687</v>
       </c>
       <c r="L152" t="s">
-        <v>695</v>
+        <v>709</v>
       </c>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>27</v>
+        <v>97</v>
       </c>
       <c r="B153" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C153">
-        <v>-57</v>
+        <v>-60.2</v>
       </c>
       <c r="D153" t="s">
         <v>587</v>
@@ -22651,16 +22737,16 @@
         <v>1</v>
       </c>
       <c r="F153" t="s">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="G153" t="b">
         <v>1</v>
       </c>
       <c r="H153" t="s">
-        <v>615</v>
+        <v>661</v>
       </c>
       <c r="I153" t="s">
-        <v>677</v>
+        <v>397</v>
       </c>
       <c r="J153" t="s">
         <v>349</v>
@@ -22669,18 +22755,18 @@
         <v>687</v>
       </c>
       <c r="L153" t="s">
-        <v>695</v>
+        <v>709</v>
       </c>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B154" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="C154">
-        <v>-7</v>
+        <v>-86</v>
       </c>
       <c r="D154" t="s">
         <v>587</v>
@@ -22689,13 +22775,13 @@
         <v>1</v>
       </c>
       <c r="F154" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="G154" t="b">
         <v>1</v>
       </c>
       <c r="H154" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="I154" t="s">
         <v>677</v>
@@ -22712,13 +22798,13 @@
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B155" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C155">
-        <v>-72</v>
+        <v>-61</v>
       </c>
       <c r="D155" t="s">
         <v>587</v>
@@ -22727,13 +22813,13 @@
         <v>1</v>
       </c>
       <c r="F155" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G155" t="b">
         <v>1</v>
       </c>
       <c r="H155" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="I155" t="s">
         <v>677</v>
@@ -22750,31 +22836,31 @@
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="B156" t="s">
-        <v>517</v>
+        <v>465</v>
       </c>
       <c r="C156">
-        <v>-500</v>
+        <v>-70</v>
       </c>
       <c r="D156" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="E156">
         <v>1</v>
       </c>
       <c r="F156" t="s">
-        <v>280</v>
+        <v>232</v>
       </c>
       <c r="G156" t="b">
         <v>1</v>
       </c>
       <c r="H156" t="s">
-        <v>653</v>
+        <v>614</v>
       </c>
       <c r="I156" t="s">
-        <v>394</v>
+        <v>677</v>
       </c>
       <c r="J156" t="s">
         <v>349</v>
@@ -22783,18 +22869,18 @@
         <v>687</v>
       </c>
       <c r="L156" t="s">
-        <v>706</v>
+        <v>695</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="B157" t="s">
-        <v>516</v>
+        <v>466</v>
       </c>
       <c r="C157">
-        <v>-170</v>
+        <v>-57</v>
       </c>
       <c r="D157" t="s">
         <v>587</v>
@@ -22803,111 +22889,263 @@
         <v>1</v>
       </c>
       <c r="F157" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="G157" t="b">
         <v>1</v>
       </c>
       <c r="H157" t="s">
-        <v>652</v>
+        <v>615</v>
       </c>
       <c r="I157" t="s">
-        <v>394</v>
+        <v>677</v>
       </c>
       <c r="J157" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="K157" t="s">
         <v>687</v>
       </c>
       <c r="L157" t="s">
-        <v>706</v>
+        <v>695</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="B158" t="s">
-        <v>518</v>
+        <v>467</v>
       </c>
       <c r="C158">
-        <v>-500</v>
+        <v>-7</v>
       </c>
       <c r="D158" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
       <c r="E158">
         <v>1</v>
       </c>
       <c r="F158" t="s">
-        <v>281</v>
+        <v>234</v>
       </c>
       <c r="G158" t="b">
         <v>1</v>
       </c>
       <c r="H158" t="s">
-        <v>653</v>
+        <v>616</v>
       </c>
       <c r="I158" t="s">
-        <v>394</v>
-      </c>
-      <c r="J158" s="2" t="s">
-        <v>356</v>
+        <v>677</v>
+      </c>
+      <c r="J158" t="s">
+        <v>349</v>
       </c>
       <c r="K158" t="s">
         <v>687</v>
       </c>
       <c r="L158" t="s">
-        <v>706</v>
+        <v>695</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
+        <v>29</v>
+      </c>
+      <c r="B159" t="s">
+        <v>468</v>
+      </c>
+      <c r="C159">
+        <v>-72</v>
+      </c>
+      <c r="D159" t="s">
+        <v>587</v>
+      </c>
+      <c r="E159">
+        <v>1</v>
+      </c>
+      <c r="F159" t="s">
+        <v>235</v>
+      </c>
+      <c r="G159" t="b">
+        <v>1</v>
+      </c>
+      <c r="H159" t="s">
+        <v>617</v>
+      </c>
+      <c r="I159" t="s">
+        <v>677</v>
+      </c>
+      <c r="J159" t="s">
+        <v>349</v>
+      </c>
+      <c r="K159" t="s">
+        <v>687</v>
+      </c>
+      <c r="L159" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
+        <v>81</v>
+      </c>
+      <c r="B160" t="s">
+        <v>517</v>
+      </c>
+      <c r="C160">
+        <v>-500</v>
+      </c>
+      <c r="D160" t="s">
+        <v>595</v>
+      </c>
+      <c r="E160">
+        <v>1</v>
+      </c>
+      <c r="F160" t="s">
+        <v>280</v>
+      </c>
+      <c r="G160" t="b">
+        <v>1</v>
+      </c>
+      <c r="H160" t="s">
+        <v>653</v>
+      </c>
+      <c r="I160" t="s">
+        <v>394</v>
+      </c>
+      <c r="J160" t="s">
+        <v>349</v>
+      </c>
+      <c r="K160" t="s">
+        <v>687</v>
+      </c>
+      <c r="L160" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
+        <v>80</v>
+      </c>
+      <c r="B161" t="s">
+        <v>516</v>
+      </c>
+      <c r="C161">
+        <v>-170</v>
+      </c>
+      <c r="D161" t="s">
+        <v>587</v>
+      </c>
+      <c r="E161">
+        <v>1</v>
+      </c>
+      <c r="F161" t="s">
+        <v>265</v>
+      </c>
+      <c r="G161" t="b">
+        <v>1</v>
+      </c>
+      <c r="H161" t="s">
+        <v>652</v>
+      </c>
+      <c r="I161" t="s">
+        <v>394</v>
+      </c>
+      <c r="J161" t="s">
+        <v>355</v>
+      </c>
+      <c r="K161" t="s">
+        <v>687</v>
+      </c>
+      <c r="L161" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
+        <v>82</v>
+      </c>
+      <c r="B162" t="s">
+        <v>518</v>
+      </c>
+      <c r="C162">
+        <v>-500</v>
+      </c>
+      <c r="D162" t="s">
+        <v>595</v>
+      </c>
+      <c r="E162">
+        <v>1</v>
+      </c>
+      <c r="F162" t="s">
+        <v>281</v>
+      </c>
+      <c r="G162" t="b">
+        <v>1</v>
+      </c>
+      <c r="H162" t="s">
+        <v>653</v>
+      </c>
+      <c r="I162" t="s">
+        <v>394</v>
+      </c>
+      <c r="J162" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="K162" t="s">
+        <v>687</v>
+      </c>
+      <c r="L162" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
         <v>14</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B163" t="s">
         <v>453</v>
       </c>
-      <c r="C159">
-        <v>1</v>
-      </c>
-      <c r="D159" t="s">
+      <c r="C163">
+        <v>1</v>
+      </c>
+      <c r="D163" t="s">
         <v>349</v>
       </c>
-      <c r="E159">
-        <v>1</v>
-      </c>
-      <c r="F159" t="s">
+      <c r="E163">
+        <v>1</v>
+      </c>
+      <c r="F163" t="s">
         <v>220</v>
       </c>
-      <c r="G159" t="b">
-        <v>1</v>
-      </c>
-      <c r="H159" t="s">
+      <c r="G163" t="b">
+        <v>1</v>
+      </c>
+      <c r="H163" t="s">
         <v>349</v>
       </c>
-      <c r="I159" t="s">
+      <c r="I163" t="s">
         <v>349</v>
       </c>
-      <c r="J159" t="s">
+      <c r="J163" t="s">
         <v>350</v>
       </c>
-      <c r="K159" t="s">
+      <c r="K163" t="s">
         <v>686</v>
       </c>
-      <c r="L159" t="s">
+      <c r="L163" t="s">
         <v>691</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L158" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L159">
-      <sortCondition ref="A1:A159"/>
+  <autoFilter ref="A1:L162" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L163">
+      <sortCondition ref="A1:A163"/>
     </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="J158" r:id="rId1" location=":~:text=Using%20the%20World%20Bank%20numbers,case%20of%20U.S.%20LMOP%20landfills." xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="J162" r:id="rId1" location=":~:text=Using%20the%20World%20Bank%20numbers,case%20of%20U.S.%20LMOP%20landfills." xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates in cost-benefits, postprocessing and Tableau
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/cb_cost_factors/cb_config_params.xlsx
+++ b/ssp_modeling/cost-benefits/cb_cost_factors/cb_config_params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_uganda_data/ssp_modeling/cost-benefits/cb_cost_factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D86C61C-F8CB-E04E-A4D4-C192C37F0926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8236CBD6-3535-2D42-B47F-9F887C324367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30780" yWindow="-9740" windowWidth="30780" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tx_table" sheetId="1" r:id="rId1"/>
@@ -6320,7 +6320,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6369,6 +6369,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -6401,7 +6407,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -6415,6 +6421,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -20105,7 +20112,7 @@
         <v>2061</v>
       </c>
       <c r="C84" s="3">
-        <v>30373</v>
+        <v>10672</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>585</v>
@@ -20135,41 +20142,41 @@
         <v>693</v>
       </c>
     </row>
-    <row r="85" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="3" t="s">
+    <row r="85" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="11" t="s">
         <v>2060</v>
       </c>
-      <c r="B85" s="3" t="s">
+      <c r="B85" s="11" t="s">
         <v>2061</v>
       </c>
-      <c r="C85" s="3">
-        <v>-135</v>
-      </c>
-      <c r="D85" s="3" t="s">
+      <c r="C85" s="11">
+        <v>-16</v>
+      </c>
+      <c r="D85" s="11" t="s">
         <v>585</v>
       </c>
-      <c r="E85" s="3">
-        <v>1</v>
-      </c>
-      <c r="F85" s="3" t="s">
+      <c r="E85" s="11">
+        <v>1</v>
+      </c>
+      <c r="F85" s="11" t="s">
         <v>2064</v>
       </c>
-      <c r="G85" s="3" t="b">
+      <c r="G85" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="H85" s="3" t="s">
+      <c r="H85" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="I85" s="3" t="s">
+      <c r="I85" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="J85" s="3" t="s">
+      <c r="J85" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="K85" s="3" t="s">
+      <c r="K85" s="11" t="s">
         <v>687</v>
       </c>
-      <c r="L85" s="3" t="s">
+      <c r="L85" s="11" t="s">
         <v>693</v>
       </c>
     </row>

</xml_diff>